<commit_message>
faster mode, class imbalance fix
</commit_message>
<xml_diff>
--- a/classifykatdpnew/kan_gat_dp_epsilo fixed long time ep4.xlsx
+++ b/classifykatdpnew/kan_gat_dp_epsilo fixed long time ep4.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\flight delay\stpn paper\STPN-main\classifykatdpnew\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB08F83B-1C26-47C5-AF70-84A3DEFB559C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FA7116-7305-4E65-8DE8-F3E03602C280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7776" yWindow="0" windowWidth="12336" windowHeight="11448"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="kan_gat_dp_epsilo fixed" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="98">
   <si>
     <t>delta</t>
   </si>
@@ -284,12 +284,42 @@
   </si>
   <si>
     <t xml:space="preserve">  12-step Departure-&gt; MAE: 3.4208, RMSE: 4.0393, R²: -0.2597</t>
+  </si>
+  <si>
+    <t>Final ε: 2.266</t>
+  </si>
+  <si>
+    <t>Final δ: 1.00e-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Precision: 1.0000 | Recall: 0.1828 | F1: 0.3091 | Accuracy: 0.1828</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  MAE: 4.1622 min | RMSE: 5.2214 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Arrival  -&gt; MAE: 5.2770, RMSE: 6.1306, R²: -0.8146</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Departure-&gt; MAE: 2.8309, RMSE: 3.7821, R²: -0.1050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Arrival  -&gt; MAE: 5.4130, RMSE: 6.2844, R²: -0.9057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Departure-&gt; MAE: 2.9089, RMSE: 3.8747, R²: -0.1591</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Arrival  -&gt; MAE: 5.5822, RMSE: 6.4608, R²: -1.0120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Departure-&gt; MAE: 2.9615, RMSE: 3.9296, R²: -0.1922</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1124,7 +1154,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L125"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1610,7 +1640,7 @@
         <v>0.62631455800000002</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1636,7 +1666,7 @@
         <v>0.61042210399999997</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1662,7 +1692,7 @@
         <v>0.58223197199999999</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1688,7 +1718,7 @@
         <v>0.58381540099999996</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1714,7 +1744,7 @@
         <v>0.55603132200000005</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1740,7 +1770,7 @@
         <v>0.54993145799999998</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1766,27 +1796,30 @@
         <v>0.52884110399999995</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L28" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="J29" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -1794,7 +1827,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>16</v>
       </c>
@@ -1802,7 +1835,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -1917,147 +1950,192 @@
         <v>29</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J49" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J50" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J53" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J54" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J56" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J57" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J59" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J60" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J61" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J62" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J63" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J64" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J65" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
three stage architecture fixed
</commit_message>
<xml_diff>
--- a/classifykatdpnew/kan_gat_dp_epsilo fixed long time ep4.xlsx
+++ b/classifykatdpnew/kan_gat_dp_epsilo fixed long time ep4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\flight delay\stpn paper\STPN-main\classifykatdpnew\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FA7116-7305-4E65-8DE8-F3E03602C280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D158A3-5590-44D3-BDB3-32A37BE323F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="177">
   <si>
     <t>delta</t>
   </si>
@@ -314,6 +314,243 @@
   </si>
   <si>
     <t xml:space="preserve">  12-step Departure-&gt; MAE: 2.9615, RMSE: 3.9296, R²: -0.1922</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Precision: 0.9881 | Recall: 0.5665 | F1: 0.7201 | Accuracy: 0.7467</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  MAE: 2.6911 min | RMSE: 3.4538 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Arrival  -&gt; MAE: 4.7942, RMSE: 5.7424, R²: -0.5921</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Departure-&gt; MAE: 1.5194, RMSE: 1.9099, R²: 0.7182</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Arrival  -&gt; MAE: 4.9344, RMSE: 5.8295, R²: -0.6398</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Departure-&gt; MAE: 1.6449, RMSE: 2.0572, R²: 0.6732</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Arrival  -&gt; MAE: 5.2821, RMSE: 6.1334, R²: -0.8133</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Departure-&gt; MAE: 2.1415, RMSE: 2.6863, R²: 0.4429</t>
+  </si>
+  <si>
+    <t>Loaded DP model from: kan_gat_dp_proper.pth</t>
+  </si>
+  <si>
+    <t>Final ε: 5.684</t>
+  </si>
+  <si>
+    <t>[INFO] Using GRAPH-LEVEL labels (MAX aggregation, ~100% delayed)</t>
+  </si>
+  <si>
+    <t>[DATA] Class distribution:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Train: 64.94% delayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Val:   23.19% delayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Test:  55.51% delayed</t>
+  </si>
+  <si>
+    <t>Auto-computed noise multiplier for target ε=20: 0.101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Sample rate: 0.0006 (batch_size=32 / total=55218)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Expected total steps: 27616 (1726 steps/epoch × 16 epochs)</t>
+  </si>
+  <si>
+    <t>Class balance (delayed): 64.94%</t>
+  </si>
+  <si>
+    <t>✓ DP-SGD enabled: ε_target=20, δ=1e-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Noise multiplier: 0.101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Sample rate: 0.0005795211706327647</t>
+  </si>
+  <si>
+    <t>Epoch 1/5 | Loss: 0.4855 | Val F1: 0.1669 | ε: 1.172/20 | Time: 1537.40s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ✓ New best checkpoint</t>
+  </si>
+  <si>
+    <t>Epoch 2/5 | Loss: 0.4578 | Val F1: 0.1135 | ε: 1.675/20 | Time: 1551.00s</t>
+  </si>
+  <si>
+    <t>Epoch 3/5 | Loss: 0.4373 | Val F1: 0.1067 | ε: 2.067/20 | Time: 1594.12s</t>
+  </si>
+  <si>
+    <t>Epoch 4/5 | Loss: 0.4352 | Val F1: 0.1066 | ε: 2.402/20 | Time: 1672.26s</t>
+  </si>
+  <si>
+    <t>Epoch 5/5 | Loss: 0.4342 | Val F1: 0.1156 | ε: 2.700/20 | Time: 1668.73s</t>
+  </si>
+  <si>
+    <t>Stage 1 completed in 8023.52s (133.73 min)</t>
+  </si>
+  <si>
+    <t>Final ε: 2.700 (target: 20)</t>
+  </si>
+  <si>
+    <t>✓ DP-SGD enabled (continuing from stage 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Current ε: 2.700 / 20</t>
+  </si>
+  <si>
+    <t>Epoch 1/11 | Train Loss: 0.1123 | Val Loss: 0.0044 | ε: 2.972/20 | Time: 1276.76s</t>
+  </si>
+  <si>
+    <t>Epoch 2/11 | Train Loss: 0.0931 | Val Loss: 0.0034 | ε: 3.225/20 | Time: 1202.38s</t>
+  </si>
+  <si>
+    <t>Epoch 3/11 | Train Loss: 0.0836 | Val Loss: 0.0031 | ε: 3.463/20 | Time: 1241.44s</t>
+  </si>
+  <si>
+    <t>Epoch 4/11 | Train Loss: 0.0800 | Val Loss: 0.0027 | ε: 3.687/20 | Time: 1246.12s</t>
+  </si>
+  <si>
+    <t>Epoch 5/11 | Train Loss: 0.0759 | Val Loss: 0.0029 | ε: 3.901/20 | Time: 1306.10s</t>
+  </si>
+  <si>
+    <t>Epoch 6/11 | Train Loss: 0.0750 | Val Loss: 0.0029 | ε: 4.106/20 | Time: 1220.98s</t>
+  </si>
+  <si>
+    <t>Epoch 7/11 | Train Loss: 0.0743 | Val Loss: 0.0031 | ε: 4.303/20 | Time: 1213.95s</t>
+  </si>
+  <si>
+    <t>Epoch 8/11 | Train Loss: 0.0715 | Val Loss: 0.0028 | ε: 4.494/20 | Time: 1195.25s</t>
+  </si>
+  <si>
+    <t>Epoch 9/11 | Train Loss: 0.0702 | Val Loss: 0.0028 | ε: 4.678/20 | Time: 1200.39s</t>
+  </si>
+  <si>
+    <t>⏹️  Early stopping triggered! No improvement for 5 epochs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Best score: 0.0027 at epoch 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Early stopping at epoch 9</t>
+  </si>
+  <si>
+    <t>Stage 2 completed in 11103.37s (185.06 min)</t>
+  </si>
+  <si>
+    <t>Final ε: 4.678 (target: 20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Precision: 0.9756 | Recall: 0.6138</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  F1: 0.7535 | Accuracy: 0.7691</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  MAE: 2.7179 min | RMSE: 3.4901 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Number of delayed samples: 9065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Target ε: 20.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Final ε: 4.678</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Train: 55218 | Val: 7871 | Test: 15763    </t>
+  </si>
+  <si>
+    <t>Final ε: 4.678</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Precision: 0.9756 | Recall: 0.6138 | F1: 0.7535 | Accuracy: 0.7691</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Arrival  -&gt; MAE: 4.8553, RMSE: 5.7870, R²: -0.6169</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Departure-&gt; MAE: 1.4850, RMSE: 1.8658, R²: 0.7311</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Arrival  -&gt; MAE: 4.9573, RMSE: 5.8360, R²: -0.6434</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Departure-&gt; MAE: 1.6372, RMSE: 2.0457, R²: 0.6769</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Arrival  -&gt; MAE: 5.3518, RMSE: 6.1864, R²: -0.8447</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Departure-&gt; MAE: 2.1537, RMSE: 2.6943, R²: 0.4395</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Precision: 0.7433 | Recall: 0.4186 | F1: 0.5356 | Accuracy: 0.4797</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  MAE: 3.4876 min | RMSE: 4.5975 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Arrival  -&gt; MAE: 3.0591, RMSE: 3.8872, R²: 0.1099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Departure-&gt; MAE: 3.9248, RMSE: 5.1192, R²: -0.3065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Arrival  -&gt; MAE: 2.9182, RMSE: 3.8404, R²: 0.1313</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Departure-&gt; MAE: 4.2101, RMSE: 5.7532, R²: -0.6501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Arrival  -&gt; MAE: 2.9693, RMSE: 4.1721, R²: -0.0253</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Departure-&gt; MAE: 4.4215, RMSE: 6.5397, R²: -1.1323</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>Final ε: 2.787</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Precision: 0.9786 | Recall: 0.6013 | F1: 0.7449 | Accuracy: 0.7632</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  MAE: 2.7182 min | RMSE: 3.4970 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Arrival  -&gt; MAE: 4.7505, RMSE: 5.7294, R²: -0.5848</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3-step Departure-&gt; MAE: 1.5018, RMSE: 1.8852, R²: 0.7255</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Arrival  -&gt; MAE: 4.9290, RMSE: 5.8242, R²: -0.6368</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6-step Departure-&gt; MAE: 1.6725, RMSE: 2.0843, R²: 0.6646</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Arrival  -&gt; MAE: 5.3722, RMSE: 6.2151, R²: -0.8619</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  12-step Departure-&gt; MAE: 2.2023, RMSE: 2.7473, R²: 0.4173</t>
   </si>
 </sst>
 </file>
@@ -1155,10 +1392,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:W207"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1196,7 +1433,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1231,7 +1468,7 @@
         <v>0.99479100499999995</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1266,7 +1503,7 @@
         <v>0.49320289699999997</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1301,7 +1538,7 @@
         <v>1.2704900000000001E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1336,7 +1573,7 @@
         <v>1.651633E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1371,7 +1608,7 @@
         <v>1.9819591000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1406,7 +1643,7 @@
         <v>0.89620124499999998</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1432,7 +1669,7 @@
         <v>0.74646165600000003</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1457,8 +1694,11 @@
       <c r="J9">
         <v>0.74151930099999996</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1483,8 +1723,11 @@
       <c r="J10">
         <v>0.727521737</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1509,8 +1752,11 @@
       <c r="J11">
         <v>0.72426341400000005</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1536,7 +1782,7 @@
         <v>0.70685970399999998</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1561,8 +1807,14 @@
       <c r="J13">
         <v>0.68652099600000005</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N13" t="s">
+        <v>15</v>
+      </c>
+      <c r="V13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1587,8 +1839,17 @@
       <c r="J14">
         <v>0.66968187599999995</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N14" t="s">
+        <v>77</v>
+      </c>
+      <c r="V14" t="s">
+        <v>77</v>
+      </c>
+      <c r="W14" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1613,8 +1874,14 @@
       <c r="J15">
         <v>0.64242973299999995</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N15" t="s">
+        <v>15</v>
+      </c>
+      <c r="V15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1640,7 +1907,7 @@
         <v>0.62631455800000002</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1665,8 +1932,14 @@
       <c r="J17">
         <v>0.61042210399999997</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N17" t="s">
+        <v>78</v>
+      </c>
+      <c r="V17" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1691,8 +1964,14 @@
       <c r="J18">
         <v>0.58223197199999999</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N18" t="s">
+        <v>152</v>
+      </c>
+      <c r="V18" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1718,7 +1997,7 @@
         <v>0.58381540099999996</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1743,8 +2022,14 @@
       <c r="J20">
         <v>0.55603132200000005</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N20" t="s">
+        <v>80</v>
+      </c>
+      <c r="V20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1769,8 +2054,14 @@
       <c r="J21">
         <v>0.54993145799999998</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N21" t="s">
+        <v>146</v>
+      </c>
+      <c r="V21" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>1.0000000000000001E-5</v>
       </c>
@@ -1796,30 +2087,78 @@
         <v>0.52884110399999995</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="N23" t="s">
+        <v>81</v>
+      </c>
+      <c r="V23" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="N24" t="s">
+        <v>153</v>
+      </c>
+      <c r="V24" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="N25" t="s">
+        <v>154</v>
+      </c>
+      <c r="V25" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N26" t="s">
+        <v>155</v>
+      </c>
+      <c r="V26" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N27" t="s">
+        <v>156</v>
+      </c>
+      <c r="V27" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>14</v>
       </c>
       <c r="L28" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N28" t="s">
+        <v>157</v>
+      </c>
+      <c r="V28" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="J29" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="N29" t="s">
+        <v>158</v>
+      </c>
+      <c r="V29" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -1827,7 +2166,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>16</v>
       </c>
@@ -1835,12 +2174,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>17</v>
       </c>
@@ -1848,7 +2187,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>18</v>
       </c>
@@ -1856,12 +2195,12 @@
         <v>79</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -1869,17 +2208,17 @@
         <v>80</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
       <c r="J37" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>21</v>
       </c>
@@ -1887,7 +2226,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>15</v>
       </c>
@@ -1895,7 +2234,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>22</v>
       </c>
@@ -1903,7 +2242,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>23</v>
       </c>
@@ -1911,7 +2250,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>24</v>
       </c>
@@ -1919,7 +2258,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>25</v>
       </c>
@@ -1927,7 +2266,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>26</v>
       </c>
@@ -1935,97 +2274,127 @@
         <v>87</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T48" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>30</v>
       </c>
       <c r="J49" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T49" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>31</v>
       </c>
       <c r="J50" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T50" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T52" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
       <c r="J53" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T53" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>34</v>
       </c>
       <c r="J54" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T54" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>36</v>
       </c>
       <c r="J56" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T56" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
       <c r="J57" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T57" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>38</v>
       </c>
       <c r="J59" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T59" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
       <c r="J60" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T60" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>15</v>
       </c>
@@ -2033,184 +2402,244 @@
         <v>93</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>39</v>
       </c>
       <c r="J62" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T62" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>15</v>
       </c>
       <c r="J63" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T63" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>22</v>
       </c>
       <c r="J64" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T64" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>40</v>
       </c>
       <c r="J65" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T65" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T66" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="T67" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J68" t="s">
+        <v>106</v>
+      </c>
+      <c r="T68" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J69" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J70" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J71" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J73" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J74" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J76" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J77" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J78" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J79" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J80" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J81" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="J82" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>28</v>
       </c>
@@ -2328,6 +2757,336 @@
     <row r="125" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>76</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A175" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="205" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="206" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="207" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>